<commit_message>
260810 before db integration
</commit_message>
<xml_diff>
--- a/chem_manager_app/dist/order book.xlsx
+++ b/chem_manager_app/dist/order book.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7387" uniqueCount="3170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7371" uniqueCount="3160">
   <si>
     <t>* 부가세(VAT) 포함 금액 기재 / 서브원 외에는 물품 "사진" 필수</t>
   </si>
@@ -9464,22 +9464,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>보관온도</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>RT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>F</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>DF</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>1</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -9492,43 +9476,19 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>35w5</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>2w5w</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>RT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>DF</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>22</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>afd</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>RT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>1</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>f</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>F</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -37291,7 +37251,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:V1044939"/>
+  <dimension ref="A1:T1044939"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="7.125" style="5" customWidth="1"/>
@@ -37310,13 +37270,11 @@
     <col min="14" max="15" width="7.625" style="1"/>
     <col min="16" max="17" width="9" style="1" customWidth="1"/>
     <col min="18" max="18" width="9.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10" style="1" customWidth="1"/>
-    <col min="20" max="20" width="7.625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="7.625" style="1"/>
-    <col min="23" max="16384" width="7.625" style="1"/>
+    <col min="19" max="19" width="7.625" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="7.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="5" customFormat="1" ht="26.25" customHeight="1">
+    <row r="1" spans="1:19" s="5" customFormat="1" ht="26.25" customHeight="1">
       <c r="A1" s="233" t="s">
         <v>2145</v>
       </c>
@@ -37333,7 +37291,7 @@
       <c r="L1" s="234"/>
       <c r="M1" s="235"/>
     </row>
-    <row r="2" spans="1:21" s="5" customFormat="1" ht="19.5" customHeight="1">
+    <row r="2" spans="1:19" s="5" customFormat="1" ht="19.5" customHeight="1">
       <c r="A2" s="225" t="s">
         <v>2146</v>
       </c>
@@ -37350,7 +37308,7 @@
       <c r="L2" s="226"/>
       <c r="M2" s="227"/>
     </row>
-    <row r="3" spans="1:21" s="5" customFormat="1" ht="27" hidden="1" customHeight="1">
+    <row r="3" spans="1:19" s="5" customFormat="1" ht="27" hidden="1" customHeight="1">
       <c r="A3" s="238" t="s">
         <v>6</v>
       </c>
@@ -37367,7 +37325,7 @@
       <c r="L3" s="219"/>
       <c r="M3" s="219"/>
     </row>
-    <row r="4" spans="1:21" s="5" customFormat="1" ht="41.25" hidden="1" customHeight="1">
+    <row r="4" spans="1:19" s="5" customFormat="1" ht="41.25" hidden="1" customHeight="1">
       <c r="A4" s="228" t="s">
         <v>2147</v>
       </c>
@@ -37384,7 +37342,7 @@
       <c r="L4" s="219"/>
       <c r="M4" s="219"/>
     </row>
-    <row r="5" spans="1:21" s="5" customFormat="1" ht="21.75" customHeight="1">
+    <row r="5" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1">
       <c r="A5" s="232" t="s">
         <v>2148</v>
       </c>
@@ -37401,7 +37359,7 @@
       <c r="L5" s="219"/>
       <c r="M5" s="219"/>
     </row>
-    <row r="6" spans="1:21" s="5" customFormat="1" ht="21.75" customHeight="1">
+    <row r="6" spans="1:19" s="5" customFormat="1" ht="21.75" customHeight="1">
       <c r="A6" s="218" t="s">
         <v>9</v>
       </c>
@@ -37418,7 +37376,7 @@
       <c r="L6" s="219"/>
       <c r="M6" s="220"/>
     </row>
-    <row r="7" spans="1:21" s="5" customFormat="1" ht="17.25" customHeight="1">
+    <row r="7" spans="1:19" s="5" customFormat="1" ht="17.25" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -37462,7 +37420,7 @@
         <v>26</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>3161</v>
+        <v>3151</v>
       </c>
       <c r="P7" s="5" t="s">
         <v>22</v>
@@ -37474,16 +37432,10 @@
         <v>23</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="T7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="5" t="s">
-        <v>3141</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    </row>
+    <row r="8" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A8" s="168" t="s">
         <v>2150</v>
       </c>
@@ -37510,7 +37462,7 @@
       <c r="L8" s="173"/>
       <c r="M8" s="174"/>
     </row>
-    <row r="9" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="9" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A9" s="168" t="s">
         <v>2153</v>
       </c>
@@ -37537,7 +37489,7 @@
       <c r="L9" s="173"/>
       <c r="M9" s="174"/>
     </row>
-    <row r="10" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="10" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A10" s="168" t="s">
         <v>2155</v>
       </c>
@@ -37564,7 +37516,7 @@
       <c r="L10" s="173"/>
       <c r="M10" s="174"/>
     </row>
-    <row r="11" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="11" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A11" s="168" t="s">
         <v>2158</v>
       </c>
@@ -37589,7 +37541,7 @@
       <c r="L11" s="173"/>
       <c r="M11" s="174"/>
     </row>
-    <row r="12" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="12" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A12" s="168" t="s">
         <v>2159</v>
       </c>
@@ -37616,7 +37568,7 @@
       <c r="L12" s="173"/>
       <c r="M12" s="174"/>
     </row>
-    <row r="13" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="13" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A13" s="168" t="s">
         <v>2161</v>
       </c>
@@ -37643,7 +37595,7 @@
       <c r="L13" s="173"/>
       <c r="M13" s="174"/>
     </row>
-    <row r="14" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="14" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A14" s="168" t="s">
         <v>2163</v>
       </c>
@@ -37669,7 +37621,7 @@
       <c r="L14" s="173"/>
       <c r="M14" s="174"/>
     </row>
-    <row r="15" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="15" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A15" s="168" t="s">
         <v>2165</v>
       </c>
@@ -37696,7 +37648,7 @@
       <c r="L15" s="173"/>
       <c r="M15" s="174"/>
     </row>
-    <row r="16" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="16" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A16" s="168" t="s">
         <v>2166</v>
       </c>
@@ -37730,11 +37682,8 @@
       <c r="O16" s="217" t="s">
         <v>2015</v>
       </c>
-      <c r="U16" s="175" t="s">
-        <v>3142</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    </row>
+    <row r="17" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A17" s="168" t="s">
         <v>2168</v>
       </c>
@@ -37761,7 +37710,7 @@
       <c r="L17" s="173"/>
       <c r="M17" s="174"/>
     </row>
-    <row r="18" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="18" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A18" s="168" t="s">
         <v>2170</v>
       </c>
@@ -37786,7 +37735,7 @@
       <c r="L18" s="173"/>
       <c r="M18" s="174"/>
     </row>
-    <row r="19" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="19" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A19" s="168" t="s">
         <v>2171</v>
       </c>
@@ -37811,7 +37760,7 @@
       <c r="L19" s="173"/>
       <c r="M19" s="174"/>
     </row>
-    <row r="20" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="20" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A20" s="168" t="s">
         <v>2172</v>
       </c>
@@ -37840,7 +37789,7 @@
       <c r="L20" s="173"/>
       <c r="M20" s="174"/>
     </row>
-    <row r="21" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="21" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A21" s="168" t="s">
         <v>2173</v>
       </c>
@@ -37886,16 +37835,10 @@
         <v>2174</v>
       </c>
       <c r="S21" s="175" t="s">
-        <v>2013</v>
-      </c>
-      <c r="T21" s="175" t="s">
         <v>2014</v>
       </c>
-      <c r="U21" s="175" t="s">
-        <v>3142</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    </row>
+    <row r="22" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A22" s="168" t="s">
         <v>2175</v>
       </c>
@@ -37939,16 +37882,10 @@
         <v>2177</v>
       </c>
       <c r="S22" s="175" t="s">
-        <v>2013</v>
-      </c>
-      <c r="T22" s="175" t="s">
         <v>2014</v>
       </c>
-      <c r="U22" s="175" t="s">
-        <v>3143</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    </row>
+    <row r="23" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A23" s="168" t="s">
         <v>2178</v>
       </c>
@@ -37975,7 +37912,7 @@
       <c r="L23" s="173"/>
       <c r="M23" s="174"/>
     </row>
-    <row r="24" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="24" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A24" s="168" t="s">
         <v>2181</v>
       </c>
@@ -38001,7 +37938,7 @@
       <c r="L24" s="173"/>
       <c r="M24" s="174"/>
     </row>
-    <row r="25" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="25" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A25" s="168" t="s">
         <v>2183</v>
       </c>
@@ -38026,7 +37963,7 @@
       <c r="L25" s="173"/>
       <c r="M25" s="174"/>
     </row>
-    <row r="26" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="26" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A26" s="168" t="s">
         <v>2186</v>
       </c>
@@ -38051,7 +37988,7 @@
       <c r="L26" s="173"/>
       <c r="M26" s="174"/>
     </row>
-    <row r="27" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="27" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A27" s="168" t="s">
         <v>2188</v>
       </c>
@@ -38076,7 +38013,7 @@
       <c r="L27" s="173"/>
       <c r="M27" s="174"/>
     </row>
-    <row r="28" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="28" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A28" s="168" t="s">
         <v>2189</v>
       </c>
@@ -38101,7 +38038,7 @@
       <c r="L28" s="173"/>
       <c r="M28" s="174"/>
     </row>
-    <row r="29" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="29" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A29" s="168" t="s">
         <v>2191</v>
       </c>
@@ -38128,7 +38065,7 @@
       <c r="L29" s="173"/>
       <c r="M29" s="174"/>
     </row>
-    <row r="30" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="30" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A30" s="168" t="s">
         <v>2192</v>
       </c>
@@ -38155,7 +38092,7 @@
       <c r="L30" s="173"/>
       <c r="M30" s="174"/>
     </row>
-    <row r="31" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="31" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A31" s="168" t="s">
         <v>2193</v>
       </c>
@@ -38182,7 +38119,7 @@
       <c r="L31" s="173"/>
       <c r="M31" s="174"/>
     </row>
-    <row r="32" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="32" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A32" s="168" t="s">
         <v>2195</v>
       </c>
@@ -38226,16 +38163,10 @@
         <v>2177</v>
       </c>
       <c r="S32" s="175" t="s">
-        <v>2013</v>
-      </c>
-      <c r="T32" s="175" t="s">
         <v>2014</v>
       </c>
-      <c r="U32" s="175" t="s">
-        <v>3144</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    </row>
+    <row r="33" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A33" s="168" t="s">
         <v>2197</v>
       </c>
@@ -38262,7 +38193,7 @@
       <c r="L33" s="173"/>
       <c r="M33" s="174"/>
     </row>
-    <row r="34" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="34" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A34" s="168" t="s">
         <v>2199</v>
       </c>
@@ -38287,7 +38218,7 @@
       <c r="L34" s="173"/>
       <c r="M34" s="174"/>
     </row>
-    <row r="35" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="35" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A35" s="168" t="s">
         <v>2200</v>
       </c>
@@ -38314,7 +38245,7 @@
       <c r="L35" s="173"/>
       <c r="M35" s="174"/>
     </row>
-    <row r="36" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="36" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A36" s="168" t="s">
         <v>2202</v>
       </c>
@@ -38341,7 +38272,7 @@
       <c r="L36" s="173"/>
       <c r="M36" s="174"/>
     </row>
-    <row r="37" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="37" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A37" s="168" t="s">
         <v>2204</v>
       </c>
@@ -38368,7 +38299,7 @@
       <c r="L37" s="173"/>
       <c r="M37" s="174"/>
     </row>
-    <row r="38" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="38" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A38" s="168" t="s">
         <v>2206</v>
       </c>
@@ -38395,7 +38326,7 @@
       <c r="L38" s="173"/>
       <c r="M38" s="174"/>
     </row>
-    <row r="39" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="39" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A39" s="168" t="s">
         <v>2208</v>
       </c>
@@ -38422,7 +38353,7 @@
       <c r="L39" s="173"/>
       <c r="M39" s="174"/>
     </row>
-    <row r="40" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="40" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A40" s="168" t="s">
         <v>2210</v>
       </c>
@@ -38457,7 +38388,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="41" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="41" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A41" s="168" t="s">
         <v>2211</v>
       </c>
@@ -38484,7 +38415,7 @@
       <c r="L41" s="173"/>
       <c r="M41" s="174"/>
     </row>
-    <row r="42" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="42" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A42" s="168" t="s">
         <v>2214</v>
       </c>
@@ -38511,7 +38442,7 @@
       <c r="L42" s="173"/>
       <c r="M42" s="174"/>
     </row>
-    <row r="43" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="43" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A43" s="168" t="s">
         <v>2215</v>
       </c>
@@ -38536,7 +38467,7 @@
       <c r="L43" s="173"/>
       <c r="M43" s="174"/>
     </row>
-    <row r="44" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="44" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A44" s="168" t="s">
         <v>2218</v>
       </c>
@@ -38563,7 +38494,7 @@
       <c r="L44" s="173"/>
       <c r="M44" s="174"/>
     </row>
-    <row r="45" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="45" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A45" s="168" t="s">
         <v>2220</v>
       </c>
@@ -38587,7 +38518,7 @@
         <v>349800</v>
       </c>
       <c r="K45" s="172" t="s">
-        <v>3145</v>
+        <v>3141</v>
       </c>
       <c r="L45" s="173"/>
       <c r="M45" s="174"/>
@@ -38598,25 +38529,19 @@
         <v>2015</v>
       </c>
       <c r="P45" s="175" t="s">
-        <v>3146</v>
+        <v>3142</v>
       </c>
       <c r="Q45" s="175">
         <v>2</v>
       </c>
       <c r="R45" s="175" t="s">
-        <v>3147</v>
+        <v>3143</v>
       </c>
       <c r="S45" s="175" t="s">
-        <v>3148</v>
-      </c>
-      <c r="T45" s="175" t="s">
-        <v>3149</v>
-      </c>
-      <c r="U45" s="175" t="s">
-        <v>3150</v>
-      </c>
-    </row>
-    <row r="46" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+        <v>3144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A46" s="168" t="s">
         <v>2222</v>
       </c>
@@ -38641,7 +38566,7 @@
       <c r="L46" s="173"/>
       <c r="M46" s="174"/>
     </row>
-    <row r="47" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="47" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A47" s="168" t="s">
         <v>2224</v>
       </c>
@@ -38665,7 +38590,7 @@
         <v>438900</v>
       </c>
       <c r="K47" s="172" t="s">
-        <v>3152</v>
+        <v>3145</v>
       </c>
       <c r="L47" s="173"/>
       <c r="M47" s="174"/>
@@ -38676,25 +38601,19 @@
         <v>2015</v>
       </c>
       <c r="P47" s="175" t="s">
-        <v>3146</v>
+        <v>3142</v>
       </c>
       <c r="Q47" s="175">
         <v>2</v>
       </c>
       <c r="R47" s="175" t="s">
-        <v>3147</v>
+        <v>3143</v>
       </c>
       <c r="S47" s="175" t="s">
-        <v>3148</v>
-      </c>
-      <c r="T47" s="175" t="s">
-        <v>3149</v>
-      </c>
-      <c r="U47" s="175" t="s">
-        <v>3151</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+        <v>3144</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A48" s="168" t="s">
         <v>2226</v>
       </c>
@@ -38721,7 +38640,7 @@
       <c r="L48" s="173"/>
       <c r="M48" s="174"/>
     </row>
-    <row r="49" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="49" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A49" s="168" t="s">
         <v>2229</v>
       </c>
@@ -38748,7 +38667,7 @@
       <c r="L49" s="173"/>
       <c r="M49" s="174"/>
     </row>
-    <row r="50" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="50" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A50" s="168" t="s">
         <v>2231</v>
       </c>
@@ -38783,7 +38702,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="51" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="51" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A51" s="168" t="s">
         <v>2234</v>
       </c>
@@ -38812,7 +38731,7 @@
       <c r="L51" s="173"/>
       <c r="M51" s="174"/>
     </row>
-    <row r="52" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="52" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A52" s="168" t="s">
         <v>2236</v>
       </c>
@@ -38847,7 +38766,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="53" spans="1:21" s="175" customFormat="1" ht="15" customHeight="1">
+    <row r="53" spans="1:19" s="175" customFormat="1" ht="15" customHeight="1">
       <c r="A53" s="168" t="s">
         <v>2238</v>
       </c>
@@ -38874,7 +38793,7 @@
       <c r="L53" s="173"/>
       <c r="M53" s="174"/>
     </row>
-    <row r="54" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="54" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A54" s="168" t="s">
         <v>2240</v>
       </c>
@@ -38899,7 +38818,7 @@
       <c r="L54" s="173"/>
       <c r="M54" s="174"/>
     </row>
-    <row r="55" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="55" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A55" s="168" t="s">
         <v>2242</v>
       </c>
@@ -38924,7 +38843,7 @@
       <c r="L55" s="173"/>
       <c r="M55" s="174"/>
     </row>
-    <row r="56" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="56" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A56" s="168" t="s">
         <v>2244</v>
       </c>
@@ -38959,7 +38878,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="57" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="57" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A57" s="180" t="s">
         <v>2246</v>
       </c>
@@ -38986,7 +38905,7 @@
       <c r="L57" s="190"/>
       <c r="M57" s="191"/>
     </row>
-    <row r="58" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="58" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A58" s="168" t="s">
         <v>2247</v>
       </c>
@@ -39013,7 +38932,7 @@
       <c r="L58" s="172"/>
       <c r="M58" s="174"/>
     </row>
-    <row r="59" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="59" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A59" s="168" t="s">
         <v>2250</v>
       </c>
@@ -39040,7 +38959,7 @@
       <c r="L59" s="172"/>
       <c r="M59" s="174"/>
     </row>
-    <row r="60" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="60" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A60" s="168" t="s">
         <v>2252</v>
       </c>
@@ -39065,7 +38984,7 @@
       <c r="L60" s="172"/>
       <c r="M60" s="174"/>
     </row>
-    <row r="61" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="61" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A61" s="168" t="s">
         <v>2253</v>
       </c>
@@ -39092,7 +39011,7 @@
       <c r="L61" s="169"/>
       <c r="M61" s="168"/>
     </row>
-    <row r="62" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="62" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A62" s="168" t="s">
         <v>2255</v>
       </c>
@@ -39119,7 +39038,7 @@
       <c r="L62" s="169"/>
       <c r="M62" s="168"/>
     </row>
-    <row r="63" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="63" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A63" s="168" t="s">
         <v>2258</v>
       </c>
@@ -39146,7 +39065,7 @@
       <c r="L63" s="169"/>
       <c r="M63" s="168"/>
     </row>
-    <row r="64" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="64" spans="1:19" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A64" s="194" t="s">
         <v>2259</v>
       </c>
@@ -39189,14 +39108,8 @@
       <c r="R64" s="175">
         <v>1</v>
       </c>
-      <c r="S64" s="175" t="s">
-        <v>3153</v>
-      </c>
-      <c r="T64" s="175">
+      <c r="S64" s="175">
         <v>1</v>
-      </c>
-      <c r="U64" s="175" t="s">
-        <v>3154</v>
       </c>
     </row>
     <row r="65" spans="1:15" s="175" customFormat="1" ht="17.25" customHeight="1">
@@ -39639,7 +39552,7 @@
       <c r="L80" s="169"/>
       <c r="M80" s="168"/>
     </row>
-    <row r="81" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="81" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A81" s="168" t="s">
         <v>2296</v>
       </c>
@@ -39666,7 +39579,7 @@
       <c r="L81" s="169"/>
       <c r="M81" s="168"/>
     </row>
-    <row r="82" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="82" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A82" s="168" t="s">
         <v>2298</v>
       </c>
@@ -39693,7 +39606,7 @@
       <c r="L82" s="169"/>
       <c r="M82" s="168"/>
     </row>
-    <row r="83" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="83" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A83" s="168" t="s">
         <v>2299</v>
       </c>
@@ -39720,7 +39633,7 @@
       <c r="L83" s="169"/>
       <c r="M83" s="168"/>
     </row>
-    <row r="84" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="84" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A84" s="168" t="s">
         <v>2301</v>
       </c>
@@ -39747,7 +39660,7 @@
       <c r="L84" s="169"/>
       <c r="M84" s="168"/>
     </row>
-    <row r="85" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="85" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A85" s="168" t="s">
         <v>2304</v>
       </c>
@@ -39771,7 +39684,7 @@
         <v>566500</v>
       </c>
       <c r="K85" s="169" t="s">
-        <v>3155</v>
+        <v>3146</v>
       </c>
       <c r="L85" s="169"/>
       <c r="M85" s="168"/>
@@ -39779,19 +39692,16 @@
         <v>2015</v>
       </c>
       <c r="O85" s="217" t="s">
-        <v>3162</v>
+        <v>3152</v>
       </c>
       <c r="Q85" s="175">
         <v>1</v>
       </c>
       <c r="R85" s="175" t="s">
-        <v>3156</v>
-      </c>
-      <c r="U85" s="175" t="s">
-        <v>3157</v>
-      </c>
-    </row>
-    <row r="86" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+        <v>3147</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A86" s="168" t="s">
         <v>2306</v>
       </c>
@@ -39818,7 +39728,7 @@
       <c r="L86" s="169"/>
       <c r="M86" s="168"/>
     </row>
-    <row r="87" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="87" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A87" s="168" t="s">
         <v>2307</v>
       </c>
@@ -39845,7 +39755,7 @@
       <c r="L87" s="169"/>
       <c r="M87" s="168"/>
     </row>
-    <row r="88" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="88" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A88" s="168" t="s">
         <v>2309</v>
       </c>
@@ -39872,7 +39782,7 @@
       <c r="L88" s="169"/>
       <c r="M88" s="168"/>
     </row>
-    <row r="89" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="89" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A89" s="168" t="s">
         <v>2311</v>
       </c>
@@ -39897,7 +39807,7 @@
       <c r="L89" s="169"/>
       <c r="M89" s="168"/>
     </row>
-    <row r="90" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="90" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A90" s="168" t="s">
         <v>2314</v>
       </c>
@@ -39924,7 +39834,7 @@
       <c r="L90" s="169"/>
       <c r="M90" s="168"/>
     </row>
-    <row r="91" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="91" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A91" s="168" t="s">
         <v>2317</v>
       </c>
@@ -39951,7 +39861,7 @@
       <c r="L91" s="169"/>
       <c r="M91" s="168"/>
     </row>
-    <row r="92" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="92" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A92" s="168" t="s">
         <v>2319</v>
       </c>
@@ -39978,7 +39888,7 @@
       <c r="L92" s="169"/>
       <c r="M92" s="168"/>
     </row>
-    <row r="93" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="93" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A93" s="168" t="s">
         <v>2320</v>
       </c>
@@ -40005,7 +39915,7 @@
       <c r="L93" s="169"/>
       <c r="M93" s="168"/>
     </row>
-    <row r="94" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="94" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A94" s="168" t="s">
         <v>2323</v>
       </c>
@@ -40032,7 +39942,7 @@
       <c r="L94" s="169"/>
       <c r="M94" s="168"/>
     </row>
-    <row r="95" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="95" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A95" s="168" t="s">
         <v>2325</v>
       </c>
@@ -40061,7 +39971,7 @@
       <c r="L95" s="169"/>
       <c r="M95" s="168"/>
     </row>
-    <row r="96" spans="1:21" s="175" customFormat="1" ht="17.25" customHeight="1">
+    <row r="96" spans="1:18" s="175" customFormat="1" ht="17.25" customHeight="1">
       <c r="A96" s="168" t="s">
         <v>2327</v>
       </c>
@@ -40436,12 +40346,12 @@
         <v>364100</v>
       </c>
       <c r="K109" s="169" t="s">
-        <v>3155</v>
+        <v>3146</v>
       </c>
       <c r="L109" s="169"/>
       <c r="M109" s="168"/>
       <c r="N109" s="217" t="s">
-        <v>3158</v>
+        <v>3148</v>
       </c>
       <c r="O109" s="217" t="s">
         <v>3139</v>
@@ -41073,12 +40983,12 @@
         <v>467500</v>
       </c>
       <c r="K132" s="169" t="s">
-        <v>3159</v>
+        <v>3149</v>
       </c>
       <c r="L132" s="169"/>
       <c r="M132" s="168"/>
       <c r="N132" s="217" t="s">
-        <v>3160</v>
+        <v>3150</v>
       </c>
       <c r="O132" s="217" t="s">
         <v>3139</v>
@@ -44523,7 +44433,7 @@
       <c r="L256" s="169"/>
       <c r="M256" s="168"/>
     </row>
-    <row r="257" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="257" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A257" s="194" t="s">
         <v>2642</v>
       </c>
@@ -44550,7 +44460,7 @@
       <c r="L257" s="169"/>
       <c r="M257" s="168"/>
     </row>
-    <row r="258" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="258" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A258" s="194" t="s">
         <v>2644</v>
       </c>
@@ -44577,11 +44487,11 @@
       <c r="N258" s="175" t="s">
         <v>1083</v>
       </c>
-      <c r="T258" s="175" t="s">
+      <c r="S258" s="175" t="s">
         <v>1083</v>
       </c>
     </row>
-    <row r="259" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="259" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A259" s="194" t="s">
         <v>2646</v>
       </c>
@@ -44606,7 +44516,7 @@
       <c r="L259" s="169"/>
       <c r="M259" s="168"/>
     </row>
-    <row r="260" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="260" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A260" s="194" t="s">
         <v>2648</v>
       </c>
@@ -44635,7 +44545,7 @@
       <c r="L260" s="169"/>
       <c r="M260" s="168"/>
     </row>
-    <row r="261" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="261" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A261" s="194" t="s">
         <v>2651</v>
       </c>
@@ -44664,7 +44574,7 @@
       <c r="L261" s="169"/>
       <c r="M261" s="168"/>
     </row>
-    <row r="262" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="262" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A262" s="194" t="s">
         <v>2653</v>
       </c>
@@ -44691,7 +44601,7 @@
       <c r="L262" s="169"/>
       <c r="M262" s="168"/>
     </row>
-    <row r="263" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="263" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A263" s="194" t="s">
         <v>2654</v>
       </c>
@@ -44718,7 +44628,7 @@
       <c r="L263" s="169"/>
       <c r="M263" s="168"/>
     </row>
-    <row r="264" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="264" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A264" s="194" t="s">
         <v>2656</v>
       </c>
@@ -44745,7 +44655,7 @@
       <c r="L264" s="169"/>
       <c r="M264" s="168"/>
     </row>
-    <row r="265" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="265" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A265" s="194" t="s">
         <v>2658</v>
       </c>
@@ -44772,7 +44682,7 @@
       <c r="L265" s="169"/>
       <c r="M265" s="168"/>
     </row>
-    <row r="266" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="266" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A266" s="194" t="s">
         <v>2660</v>
       </c>
@@ -44801,7 +44711,7 @@
       <c r="L266" s="169"/>
       <c r="M266" s="168"/>
     </row>
-    <row r="267" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="267" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A267" s="194" t="s">
         <v>2662</v>
       </c>
@@ -44826,7 +44736,7 @@
       <c r="L267" s="169"/>
       <c r="M267" s="168"/>
     </row>
-    <row r="268" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="268" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A268" s="194" t="s">
         <v>2665</v>
       </c>
@@ -44853,7 +44763,7 @@
       <c r="L268" s="169"/>
       <c r="M268" s="168"/>
     </row>
-    <row r="269" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="269" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A269" s="194" t="s">
         <v>2667</v>
       </c>
@@ -44880,7 +44790,7 @@
       <c r="L269" s="169"/>
       <c r="M269" s="168"/>
     </row>
-    <row r="270" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="270" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A270" s="194" t="s">
         <v>2668</v>
       </c>
@@ -44907,7 +44817,7 @@
       <c r="L270" s="169"/>
       <c r="M270" s="168"/>
     </row>
-    <row r="271" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="271" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A271" s="194" t="s">
         <v>2669</v>
       </c>
@@ -44934,7 +44844,7 @@
       <c r="L271" s="169"/>
       <c r="M271" s="168"/>
     </row>
-    <row r="272" spans="1:20" s="175" customFormat="1" ht="16.5" customHeight="1">
+    <row r="272" spans="1:19" s="175" customFormat="1" ht="16.5" customHeight="1">
       <c r="A272" s="194" t="s">
         <v>2670</v>
       </c>
@@ -50207,10 +50117,10 @@
       <c r="L462" s="169"/>
       <c r="M462" s="168"/>
       <c r="N462" s="217" t="s">
-        <v>3163</v>
+        <v>3153</v>
       </c>
       <c r="O462" s="217" t="s">
-        <v>3163</v>
+        <v>3153</v>
       </c>
     </row>
     <row r="463" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50487,10 +50397,10 @@
       <c r="L472" s="169"/>
       <c r="M472" s="168"/>
       <c r="N472" s="217" t="s">
-        <v>3164</v>
+        <v>3154</v>
       </c>
       <c r="O472" s="217" t="s">
-        <v>3164</v>
+        <v>3154</v>
       </c>
     </row>
     <row r="473" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50547,10 +50457,10 @@
       <c r="L474" s="169"/>
       <c r="M474" s="168"/>
       <c r="N474" s="217" t="s">
-        <v>3168</v>
+        <v>3158</v>
       </c>
       <c r="O474" s="217" t="s">
-        <v>3168</v>
+        <v>3158</v>
       </c>
     </row>
     <row r="475" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50578,10 +50488,10 @@
       <c r="L475" s="169"/>
       <c r="M475" s="168"/>
       <c r="N475" s="217" t="s">
-        <v>3169</v>
+        <v>3159</v>
       </c>
       <c r="O475" s="217" t="s">
-        <v>3169</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="476" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50611,10 +50521,10 @@
       <c r="L476" s="169"/>
       <c r="M476" s="168"/>
       <c r="N476" s="217" t="s">
-        <v>3166</v>
+        <v>3156</v>
       </c>
       <c r="O476" s="217" t="s">
-        <v>3166</v>
+        <v>3156</v>
       </c>
     </row>
     <row r="477" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50673,10 +50583,10 @@
       <c r="L478" s="169"/>
       <c r="M478" s="168"/>
       <c r="N478" s="217" t="s">
-        <v>3167</v>
+        <v>3157</v>
       </c>
       <c r="O478" s="217" t="s">
-        <v>3167</v>
+        <v>3157</v>
       </c>
     </row>
     <row r="479" spans="1:15" s="175" customFormat="1" ht="16.5" customHeight="1">
@@ -50733,10 +50643,10 @@
       <c r="L480" s="169"/>
       <c r="M480" s="168"/>
       <c r="N480" s="217" t="s">
-        <v>3165</v>
+        <v>3155</v>
       </c>
       <c r="O480" s="217" t="s">
-        <v>3165</v>
+        <v>3155</v>
       </c>
     </row>
     <row r="481" spans="1:13" s="175" customFormat="1" ht="16.5" customHeight="1">

</xml_diff>

<commit_message>
260812 with db before onedrive-compatible-patch
</commit_message>
<xml_diff>
--- a/chem_manager_app/dist/order book.xlsx
+++ b/chem_manager_app/dist/order book.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7371" uniqueCount="3160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7374" uniqueCount="3161">
   <si>
     <t>* 부가세(VAT) 포함 금액 기재 / 서브원 외에는 물품 "사진" 필수</t>
   </si>
@@ -9537,6 +9537,10 @@
   </si>
   <si>
     <t>O</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>aldrich</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -46647,7 +46651,7 @@
       <c r="L336" s="169"/>
       <c r="M336" s="168"/>
     </row>
-    <row r="337" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="337" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A337" s="194" t="s">
         <v>2798</v>
       </c>
@@ -46676,7 +46680,7 @@
       <c r="L337" s="169"/>
       <c r="M337" s="168"/>
     </row>
-    <row r="338" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="338" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A338" s="194" t="s">
         <v>2800</v>
       </c>
@@ -46703,7 +46707,7 @@
       <c r="L338" s="169"/>
       <c r="M338" s="168"/>
     </row>
-    <row r="339" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="339" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A339" s="194" t="s">
         <v>2801</v>
       </c>
@@ -46730,7 +46734,7 @@
       <c r="L339" s="169"/>
       <c r="M339" s="168"/>
     </row>
-    <row r="340" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="340" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A340" s="194" t="s">
         <v>2802</v>
       </c>
@@ -46757,7 +46761,7 @@
       <c r="L340" s="169"/>
       <c r="M340" s="168"/>
     </row>
-    <row r="341" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="341" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A341" s="194" t="s">
         <v>2804</v>
       </c>
@@ -46784,7 +46788,7 @@
       <c r="L341" s="169"/>
       <c r="M341" s="168"/>
     </row>
-    <row r="342" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="342" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A342" s="194" t="s">
         <v>2806</v>
       </c>
@@ -46811,7 +46815,7 @@
       <c r="L342" s="169"/>
       <c r="M342" s="168"/>
     </row>
-    <row r="343" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="343" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A343" s="194" t="s">
         <v>2808</v>
       </c>
@@ -46838,7 +46842,7 @@
       <c r="L343" s="169"/>
       <c r="M343" s="168"/>
     </row>
-    <row r="344" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="344" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A344" s="194" t="s">
         <v>2810</v>
       </c>
@@ -46867,7 +46871,7 @@
       <c r="L344" s="169"/>
       <c r="M344" s="168"/>
     </row>
-    <row r="345" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="345" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A345" s="194" t="s">
         <v>2812</v>
       </c>
@@ -46896,7 +46900,7 @@
       <c r="L345" s="169"/>
       <c r="M345" s="168"/>
     </row>
-    <row r="346" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="346" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A346" s="194" t="s">
         <v>2814</v>
       </c>
@@ -46925,7 +46929,7 @@
       <c r="L346" s="169"/>
       <c r="M346" s="168"/>
     </row>
-    <row r="347" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="347" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A347" s="194" t="s">
         <v>2816</v>
       </c>
@@ -46953,8 +46957,26 @@
       <c r="K347" s="169"/>
       <c r="L347" s="169"/>
       <c r="M347" s="168"/>
-    </row>
-    <row r="348" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+      <c r="N347" s="175" t="s">
+        <v>3139</v>
+      </c>
+      <c r="O347" s="175" t="s">
+        <v>3139</v>
+      </c>
+      <c r="P347" s="175" t="s">
+        <v>3160</v>
+      </c>
+      <c r="Q347" s="175">
+        <v>1</v>
+      </c>
+      <c r="R347" s="175">
+        <v>50</v>
+      </c>
+      <c r="S347" s="175">
+        <v>402788</v>
+      </c>
+    </row>
+    <row r="348" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A348" s="194" t="s">
         <v>2818</v>
       </c>
@@ -46983,7 +47005,7 @@
       <c r="L348" s="169"/>
       <c r="M348" s="168"/>
     </row>
-    <row r="349" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="349" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A349" s="194" t="s">
         <v>2820</v>
       </c>
@@ -47012,7 +47034,7 @@
       <c r="L349" s="169"/>
       <c r="M349" s="168"/>
     </row>
-    <row r="350" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="350" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A350" s="194" t="s">
         <v>2822</v>
       </c>
@@ -47037,7 +47059,7 @@
       <c r="L350" s="169"/>
       <c r="M350" s="168"/>
     </row>
-    <row r="351" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="351" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A351" s="194" t="s">
         <v>2824</v>
       </c>
@@ -47062,7 +47084,7 @@
       <c r="L351" s="169"/>
       <c r="M351" s="168"/>
     </row>
-    <row r="352" spans="1:13" s="175" customFormat="1" ht="15.75" customHeight="1">
+    <row r="352" spans="1:19" s="175" customFormat="1" ht="15.75" customHeight="1">
       <c r="A352" s="194" t="s">
         <v>2826</v>
       </c>

</xml_diff>